<commit_message>
Expand tax workbook with full Canada-wide tax system sheets
Adds five sheets to personal_tax_outline_2026.xlsx: all 14
jurisdictions' income tax brackets and basic personal amounts, sales
tax rates, full payroll contribution parameters (CPP/CPP2/QPP/EI/QPIP),
corporate tax rates, and credits/limits — all generated from the
data/json dataset alongside the existing personal calculation.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ehz8TwmzopJMrdk2ad5vgV
</commit_message>
<xml_diff>
--- a/examples/personal_tax_outline_2026.xlsx
+++ b/examples/personal_tax_outline_2026.xlsx
@@ -11,6 +11,11 @@
     <sheet name="Inputs" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Tax Data 2026" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Tax Calc" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="All Income Brackets" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Sales Tax" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Payroll CPP EI" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Corporate Tax" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Credits &amp; Limits" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -150,7 +155,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="186">
   <si>
     <t xml:space="preserve">2026 Tax Outline — Inputs</t>
   </si>
@@ -414,18 +419,314 @@
   </si>
   <si>
     <t xml:space="preserve">Notes: 2026 rules, Alberta resident, single filer, no other income/deductions. Employer withholding assumed to cover the salary-only liability. No EI on self-employment income (opt-in not assumed). Estimates for planning, not filing — see docs/trader_taxation.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personal Income Tax Brackets 2026 — All of Canada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Federal + every province/territory. Source: data/json/personal_income_tax_2026.json (CRA figures; see README.md).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jurisdiction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bracket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marginal rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canada (federal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alberta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">British Columbia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saskatchewan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manitoba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ontario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quebec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New Brunswick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nova Scotia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prince Edward Island</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Newfoundland and Labrador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yukon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Northwest Territories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nunavut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basic personal amounts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phases down to $14,829 for income above $181,440</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n/a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sales Tax Rates 2026 — GST / HST / PST / QST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: data/json/sales_tax_2026.json.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Province/Territory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PST/QST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GST + PST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GST + RST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GST + QST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HST reduced from 15% to 14% effective April 1, 2025.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payroll Contributions 2026 — CPP, CPP2, QPP, EI, QPIP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: data/json/payroll_contributions_2026.json.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canada Pension Plan (base + first additional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ympe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">basic exemption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">employee rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">employer rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">self employed rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max employee contribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max self employed contribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YMPE (Year's Maximum Pensionable Earnings) rose from $71,300 in 2025 to $74,600 in 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPP second additional contribution (CPP2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yampe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applies to pensionable earnings between the YMPE and the YAMPE (Year's Additional Maximum Pensionable Earnings, $85,000 in 2026, up from $81,200 in 2025).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quebec Pension Plan (base + first additional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qpp2 rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quebec reduced the QPP first-tier rate to 6.30% for 2026 (it was 6.40% in 2025). QPP2 mirrors CPP2 at 4% on the YMPE-YAMPE band.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Employment Insurance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maximum insurable earnings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">employer rate multiplier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max employee premium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max employer premium per employee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quebec employee rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quebec employer rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quebec max employee premium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum insurable earnings rose from $65,700 in 2025 to $68,900 in 2026; the employee rate is $1.63 per $100 of insurable earnings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quebec Parental Insurance Plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QPIP premium rates fell for 2026 (employee rate from 0.494% to 0.430%) while the insurable earnings maximum rose to $103,000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corporate Income Tax Rates 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: data/json/corporate_income_tax_2026.json.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small business rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SB limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saskatchewan's 1% small-business rate was made permanent in 2025; its business limit is $600,000, the only province above $500,000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small-business rate reduced from 3.2% to 2.2% for taxation years beginning on or after July 1, 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small-business rate reduced from 3.2% to 2.2% for taxation years beginning after April 29, 2026. Quebec's small-business rate requires minimum employee paid-hours; corporations that do not qualify pay the general rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General rate cut from 16% to 14% and small-business rate from 2.5% to 1.5% effective April 1, 2025.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small-business rate reduced from 2.5% to 2.0% effective January 1, 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Key Credits, Registered Accounts &amp; System Parameters 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: data/json/credits_and_limits_2026.json.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TFSA annual limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumulative room applies to someone 18+ in 2009 who has never contributed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TFSA cumulative room since 2009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RRSP annual limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18% of previous year's earned income, up to the annual limit; unused room carries forward indefinitely.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FHSA annual limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum single-year contribution is $16,000 ($8,000 annual + $8,000 carried forward).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FHSA lifetime limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Federal BPA (max)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Federal BPA (min, high income)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Federal credit rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Federal non-refundable credits are valued at the lowest federal rate (14% in 2026). Provincial credits use each province's lowest rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OAS clawback threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OAS recovery tax: 15% of net income above the threshold for the 2026 income year.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OAS recovery rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capital gains inclusion rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proposed increase to a 2/3 inclusion rate was cancelled in March 2025; the rate remains 50%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lifetime capital gains exemption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quebec abatement rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trading note: for an active/scalp trader, profits are business income — the capital gains inclusion rate does not apply. See docs/trader_taxation.md.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="168" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
+    <numFmt numFmtId="169" formatCode="0.00%"/>
+    <numFmt numFmtId="170" formatCode="0.000%"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -573,7 +874,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -668,6 +969,14 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2217,4 +2526,2434 @@
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E89"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>58523</v>
+      </c>
+      <c r="E5" s="24" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>58523</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>117045</v>
+      </c>
+      <c r="E6" s="24" t="n">
+        <v>0.205</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>117045</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>181440</v>
+      </c>
+      <c r="E7" s="24" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>181440</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>258482</v>
+      </c>
+      <c r="E8" s="24" t="n">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>258482</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E9" s="24" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>61200</v>
+      </c>
+      <c r="E10" s="24" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>61200</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>151234</v>
+      </c>
+      <c r="E11" s="24" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>151234</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>181480</v>
+      </c>
+      <c r="E12" s="24" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>181480</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>241975</v>
+      </c>
+      <c r="E13" s="24" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>241975</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>362962</v>
+      </c>
+      <c r="E14" s="24" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>362962</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" s="24" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>50363</v>
+      </c>
+      <c r="E16" s="24" t="n">
+        <v>0.056</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>50363</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>100728</v>
+      </c>
+      <c r="E17" s="24" t="n">
+        <v>0.077</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>100728</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>115647</v>
+      </c>
+      <c r="E18" s="24" t="n">
+        <v>0.105</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>115647</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>140430</v>
+      </c>
+      <c r="E19" s="24" t="n">
+        <v>0.1229</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>140430</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>190405</v>
+      </c>
+      <c r="E20" s="24" t="n">
+        <v>0.147</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>190405</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>265545</v>
+      </c>
+      <c r="E21" s="24" t="n">
+        <v>0.168</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>265545</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E22" s="24" t="n">
+        <v>0.205</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>54532</v>
+      </c>
+      <c r="E23" s="24" t="n">
+        <v>0.105</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>54532</v>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>155805</v>
+      </c>
+      <c r="E24" s="24" t="n">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>155805</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E25" s="24" t="n">
+        <v>0.145</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>47564</v>
+      </c>
+      <c r="E26" s="24" t="n">
+        <v>0.108</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>47564</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>101200</v>
+      </c>
+      <c r="E27" s="24" t="n">
+        <v>0.1275</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>101200</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E28" s="24" t="n">
+        <v>0.174</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>53891</v>
+      </c>
+      <c r="E29" s="24" t="n">
+        <v>0.0505</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>53891</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>107785</v>
+      </c>
+      <c r="E30" s="24" t="n">
+        <v>0.0915</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>107785</v>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>150000</v>
+      </c>
+      <c r="E31" s="24" t="n">
+        <v>0.1116</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>220000</v>
+      </c>
+      <c r="E32" s="24" t="n">
+        <v>0.1216</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>220000</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E33" s="24" t="n">
+        <v>0.1316</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>54345</v>
+      </c>
+      <c r="E34" s="24" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" s="9" t="n">
+        <v>54345</v>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>108680</v>
+      </c>
+      <c r="E35" s="24" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" s="9" t="n">
+        <v>108680</v>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>132245</v>
+      </c>
+      <c r="E36" s="24" t="n">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" s="9" t="n">
+        <v>132245</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E37" s="24" t="n">
+        <v>0.2575</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="9" t="n">
+        <v>52332</v>
+      </c>
+      <c r="E38" s="24" t="n">
+        <v>0.094</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B39" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" s="9" t="n">
+        <v>52332</v>
+      </c>
+      <c r="D39" s="9" t="n">
+        <v>104666</v>
+      </c>
+      <c r="E39" s="24" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C40" s="9" t="n">
+        <v>104666</v>
+      </c>
+      <c r="D40" s="9" t="n">
+        <v>193861</v>
+      </c>
+      <c r="E40" s="24" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B41" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C41" s="9" t="n">
+        <v>193861</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E41" s="24" t="n">
+        <v>0.195</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="9" t="n">
+        <v>30995</v>
+      </c>
+      <c r="E42" s="24" t="n">
+        <v>0.0879</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B43" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" s="9" t="n">
+        <v>30995</v>
+      </c>
+      <c r="D43" s="9" t="n">
+        <v>61991</v>
+      </c>
+      <c r="E43" s="24" t="n">
+        <v>0.1495</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B44" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C44" s="9" t="n">
+        <v>61991</v>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>97417</v>
+      </c>
+      <c r="E44" s="24" t="n">
+        <v>0.1667</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B45" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C45" s="9" t="n">
+        <v>97417</v>
+      </c>
+      <c r="D45" s="9" t="n">
+        <v>157124</v>
+      </c>
+      <c r="E45" s="24" t="n">
+        <v>0.175</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B46" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C46" s="9" t="n">
+        <v>157124</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E46" s="24" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>33928</v>
+      </c>
+      <c r="E47" s="24" t="n">
+        <v>0.095</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B48" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" s="9" t="n">
+        <v>33928</v>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>65820</v>
+      </c>
+      <c r="E48" s="24" t="n">
+        <v>0.1347</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B49" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C49" s="9" t="n">
+        <v>65820</v>
+      </c>
+      <c r="D49" s="9" t="n">
+        <v>106890</v>
+      </c>
+      <c r="E49" s="24" t="n">
+        <v>0.166</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B50" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C50" s="9" t="n">
+        <v>106890</v>
+      </c>
+      <c r="D50" s="9" t="n">
+        <v>142520</v>
+      </c>
+      <c r="E50" s="24" t="n">
+        <v>0.1762</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B51" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C51" s="9" t="n">
+        <v>142520</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E51" s="24" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="9" t="n">
+        <v>44678</v>
+      </c>
+      <c r="E52" s="24" t="n">
+        <v>0.087</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B53" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" s="9" t="n">
+        <v>44678</v>
+      </c>
+      <c r="D53" s="9" t="n">
+        <v>89354</v>
+      </c>
+      <c r="E53" s="24" t="n">
+        <v>0.145</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B54" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" s="9" t="n">
+        <v>89354</v>
+      </c>
+      <c r="D54" s="9" t="n">
+        <v>159528</v>
+      </c>
+      <c r="E54" s="24" t="n">
+        <v>0.158</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B55" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C55" s="9" t="n">
+        <v>159528</v>
+      </c>
+      <c r="D55" s="9" t="n">
+        <v>223340</v>
+      </c>
+      <c r="E55" s="24" t="n">
+        <v>0.178</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B56" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C56" s="9" t="n">
+        <v>223340</v>
+      </c>
+      <c r="D56" s="9" t="n">
+        <v>285319</v>
+      </c>
+      <c r="E56" s="24" t="n">
+        <v>0.198</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B57" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C57" s="9" t="n">
+        <v>285319</v>
+      </c>
+      <c r="D57" s="9" t="n">
+        <v>570638</v>
+      </c>
+      <c r="E57" s="24" t="n">
+        <v>0.208</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B58" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C58" s="9" t="n">
+        <v>570638</v>
+      </c>
+      <c r="D58" s="9" t="n">
+        <v>1141275</v>
+      </c>
+      <c r="E58" s="24" t="n">
+        <v>0.213</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B59" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C59" s="9" t="n">
+        <v>1141275</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E59" s="24" t="n">
+        <v>0.218</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B60" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" s="9" t="n">
+        <v>58523</v>
+      </c>
+      <c r="E60" s="24" t="n">
+        <v>0.064</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B61" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C61" s="9" t="n">
+        <v>58523</v>
+      </c>
+      <c r="D61" s="9" t="n">
+        <v>117045</v>
+      </c>
+      <c r="E61" s="24" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B62" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C62" s="9" t="n">
+        <v>117045</v>
+      </c>
+      <c r="D62" s="9" t="n">
+        <v>181440</v>
+      </c>
+      <c r="E62" s="24" t="n">
+        <v>0.109</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B63" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C63" s="9" t="n">
+        <v>181440</v>
+      </c>
+      <c r="D63" s="9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E63" s="24" t="n">
+        <v>0.128</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B64" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C64" s="9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E64" s="24" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B65" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="9" t="n">
+        <v>53003</v>
+      </c>
+      <c r="E65" s="24" t="n">
+        <v>0.059</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B66" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" s="9" t="n">
+        <v>53003</v>
+      </c>
+      <c r="D66" s="9" t="n">
+        <v>106009</v>
+      </c>
+      <c r="E66" s="24" t="n">
+        <v>0.086</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B67" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" s="9" t="n">
+        <v>106009</v>
+      </c>
+      <c r="D67" s="9" t="n">
+        <v>172346</v>
+      </c>
+      <c r="E67" s="24" t="n">
+        <v>0.122</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B68" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" s="9" t="n">
+        <v>172346</v>
+      </c>
+      <c r="D68" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E68" s="24" t="n">
+        <v>0.1405</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B69" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="9" t="n">
+        <v>55801</v>
+      </c>
+      <c r="E69" s="24" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B70" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C70" s="9" t="n">
+        <v>55801</v>
+      </c>
+      <c r="D70" s="9" t="n">
+        <v>111601</v>
+      </c>
+      <c r="E70" s="24" t="n">
+        <v>0.07</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B71" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C71" s="9" t="n">
+        <v>111601</v>
+      </c>
+      <c r="D71" s="9" t="n">
+        <v>181439</v>
+      </c>
+      <c r="E71" s="24" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B72" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C72" s="9" t="n">
+        <v>181439</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E72" s="24" t="n">
+        <v>0.115</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B76" s="9" t="n">
+        <v>16452</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B77" s="9" t="n">
+        <v>22769</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B78" s="9" t="n">
+        <v>13217</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B79" s="9" t="n">
+        <v>19371</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B80" s="9" t="n">
+        <v>15780</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B81" s="9" t="n">
+        <v>12989</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B82" s="9" t="n">
+        <v>18952</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B83" s="9" t="n">
+        <v>13664</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B84" s="9" t="n">
+        <v>11932</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B85" s="9" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B86" s="9" t="n">
+        <v>11189</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B87" s="9" t="n">
+        <v>16452</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B88" s="9" t="n">
+        <v>18199</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B89" s="9" t="n">
+        <v>19659</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" s="24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="F5" s="24" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" s="24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D6" s="24" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="E6" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="F6" s="24" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C7" s="24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D7" s="24" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="F7" s="24" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C8" s="24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D8" s="24" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="F8" s="24" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="E9" s="24" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F9" s="24" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C10" s="24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D10" s="24" t="n">
+        <v>0.09975</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="F10" s="24" t="n">
+        <v>0.14975</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="E11" s="24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F11" s="24" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="E12" s="24" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="F12" s="24" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="E13" s="24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F13" s="24" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="E14" s="24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F14" s="24" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C15" s="24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="F15" s="24" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C16" s="24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D16" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="F16" s="24" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C17" s="24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="F17" s="24" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B50"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="70"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" s="12"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>74600</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" s="25" t="n">
+        <v>0.0595</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" s="25" t="n">
+        <v>0.0595</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B9" s="25" t="n">
+        <v>0.119</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B10" s="19" t="n">
+        <v>4230.45</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B11" s="19" t="n">
+        <v>8460.9</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="B14" s="12"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B16" s="25" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="25" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B18" s="25" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B19" s="19" t="n">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B20" s="19" t="n">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="B23" s="12"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B24" s="19" t="n">
+        <v>74600</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B25" s="19" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B26" s="25" t="n">
+        <v>0.063</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B27" s="25" t="n">
+        <v>0.063</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28" s="19" t="n">
+        <v>4479.3</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B29" s="25" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B32" s="12"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B33" s="19" t="n">
+        <v>68900</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B34" s="25" t="n">
+        <v>0.0163</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B35" s="19" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B36" s="25" t="n">
+        <v>0.02282</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B37" s="19" t="n">
+        <v>1123.07</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B38" s="19" t="n">
+        <v>1572.3</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B39" s="25" t="n">
+        <v>0.013</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B40" s="25" t="n">
+        <v>0.0182</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B41" s="19" t="n">
+        <v>895.7</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="B44" s="12"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B45" s="19" t="n">
+        <v>103000</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B46" s="25" t="n">
+        <v>0.0043</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B47" s="25" t="n">
+        <v>0.00602</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B48" s="19" t="n">
+        <v>442.9</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B49" s="19" t="n">
+        <v>620.06</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6" t="s">
+        <v>152</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="70"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>600000</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="70"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>109000</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>33810</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>16452</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>14829</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>95323</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>1250000</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>0.165</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>185</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>